<commit_message>
Fix critical rendering issues and complete Récapitulatif structure
- Fix fill alpha: all PatternFill now use FF prefix (colors were transparent)
- Fix Paramètres H formula: use ="" to detect empty cells (matches reference)
- Add poste reference table in Paramètres (IFERROR/MID formulas linked to Récapitulatif)
- Add TOTAL NON RÉCUPÉRABLES and TOTAL GÉNÉRAL rows at end of Récapitulatif
- Fix Vacance Locative cost formula: use D-F instead of D*(1-H/365)
- Rename F6 header in Paramètres from "Début de bail / MAD" to "Début de bail"

https://claude.ai/code/session_016DCHgeFEbekAwEc4Sro4Qi
</commit_message>
<xml_diff>
--- a/regularisation_ORMES_A_2025.xlsx
+++ b/regularisation_ORMES_A_2025.xlsx
@@ -28,7 +28,7 @@
     <numFmt numFmtId="168" formatCode="0.0000"/>
     <numFmt numFmtId="169" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -78,7 +78,18 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="00000000"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00444444"/>
       <sz val="9"/>
     </font>
     <font>
@@ -91,12 +102,6 @@
       <name val="Calibri"/>
       <color rgb="00222222"/>
       <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -119,37 +124,37 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001B3A6B"/>
+        <fgColor rgb="FF1B3A6B"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D0DDEF"/>
+        <fgColor rgb="FFD0DDEF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002E5FA3"/>
+        <fgColor rgb="FF2E5FA3"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F4F8"/>
+        <fgColor rgb="FFF2F4F8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D5F5E3"/>
+        <fgColor rgb="FFD5F5E3"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FDECEA"/>
+        <fgColor rgb="FFFDECEA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E64A19"/>
+        <fgColor rgb="FFE64A19"/>
       </patternFill>
     </fill>
   </fills>
@@ -165,7 +170,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -204,10 +209,19 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -222,19 +236,31 @@
     <xf numFmtId="166" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -247,33 +273,21 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -285,10 +299,10 @@
     <xf numFmtId="164" fontId="4" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="14" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="169" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -659,7 +673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G118"/>
+  <dimension ref="A1:G122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3248,8 +3262,33 @@
         <v/>
       </c>
     </row>
+    <row r="119" ht="6" customHeight="1"/>
+    <row r="120" ht="19.55" customHeight="1">
+      <c r="A120" s="5" t="inlineStr">
+        <is>
+          <t>TOTAL — CHARGES NON RÉCUPÉRABLES</t>
+        </is>
+      </c>
+      <c r="E120" s="14">
+        <f>E118</f>
+        <v/>
+      </c>
+    </row>
+    <row r="121" ht="6" customHeight="1"/>
+    <row r="122" ht="25.55" customHeight="1">
+      <c r="A122" s="15" t="inlineStr">
+        <is>
+          <t>TOTAL GÉNÉRAL — CHARGES RÉCUPÉRABLES</t>
+        </is>
+      </c>
+      <c r="E122" s="16">
+        <f>E10+E21+E32+E37+E46+E50+E54+E59+E64+E77+E83+E88+E97+E101+E104+E107+E111</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="25">
+  <mergeCells count="27">
+    <mergeCell ref="A122:D122"/>
     <mergeCell ref="A97:D97"/>
     <mergeCell ref="A4:G4"/>
     <mergeCell ref="A38:G38"/>
@@ -3268,6 +3307,7 @@
     <mergeCell ref="A46:D46"/>
     <mergeCell ref="A118:D118"/>
     <mergeCell ref="A37:D37"/>
+    <mergeCell ref="A120:D120"/>
     <mergeCell ref="A50:D50"/>
     <mergeCell ref="A101:D101"/>
     <mergeCell ref="A21:D21"/>
@@ -3286,7 +3326,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3313,7 +3353,7 @@
           <t>Site</t>
         </is>
       </c>
-      <c r="C2" s="14" t="inlineStr">
+      <c r="C2" s="17" t="inlineStr">
         <is>
           <t>ORMES A</t>
         </is>
@@ -3325,7 +3365,7 @@
           <t>Surface totale site (m²)</t>
         </is>
       </c>
-      <c r="C3" s="14" t="n">
+      <c r="C3" s="17" t="n">
         <v>29565.91</v>
       </c>
     </row>
@@ -3335,7 +3375,7 @@
           <t>Année</t>
         </is>
       </c>
-      <c r="C4" s="14" t="n">
+      <c r="C4" s="17" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -3368,7 +3408,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Début de bail / MAD</t>
+          <t>Début de bail</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -3388,70 +3428,264 @@
       </c>
     </row>
     <row r="7" ht="15.05" customHeight="1">
-      <c r="A7" s="14" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>C1 C2</t>
         </is>
       </c>
-      <c r="B7" s="15" t="inlineStr">
+      <c r="B7" s="18" t="inlineStr">
         <is>
           <t>Occupé</t>
         </is>
       </c>
-      <c r="C7" s="16" t="n">
+      <c r="C7" s="19" t="n">
         <v>9623</v>
       </c>
-      <c r="D7" s="17" t="inlineStr"/>
-      <c r="E7" s="18" t="inlineStr">
+      <c r="D7" s="20" t="inlineStr"/>
+      <c r="E7" s="21" t="inlineStr">
         <is>
           <t>ID LOGISTICS</t>
         </is>
       </c>
-      <c r="F7" s="19" t="n">
+      <c r="F7" s="22" t="n">
         <v>45737</v>
       </c>
-      <c r="G7" s="19" t="n">
+      <c r="G7" s="22" t="n">
         <v>50119</v>
       </c>
-      <c r="H7" s="20">
-        <f>MAX(0,MIN(DATE(2025,12,31),IF(G7&gt;0,G7,DATE(2025,12,31)))-MAX(DATE(2025,1,1),IF(F7&gt;0,F7,DATE(2025,1,1)))+1)</f>
-        <v/>
-      </c>
-      <c r="I7" s="21">
+      <c r="H7" s="23">
+        <f>MAX(0,MIN(DATE(2025,12,31),IF(G7="",DATE(2025,12,31),G7))-MAX(DATE(2025,1,1),IF(F7="",DATE(2025,1,1),F7))+1)</f>
+        <v/>
+      </c>
+      <c r="I7" s="24">
         <f>H7/365</f>
         <v/>
       </c>
     </row>
     <row r="8" ht="15.05" customHeight="1">
-      <c r="A8" s="14" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>C3 C4 C5</t>
         </is>
       </c>
-      <c r="B8" s="22" t="inlineStr">
+      <c r="B8" s="25" t="inlineStr">
         <is>
           <t>Vacant</t>
         </is>
       </c>
-      <c r="C8" s="16" t="n">
+      <c r="C8" s="19" t="n">
         <v>19942.91</v>
       </c>
-      <c r="D8" s="17" t="inlineStr"/>
-      <c r="E8" s="18" t="inlineStr"/>
-      <c r="F8" s="17" t="n"/>
-      <c r="G8" s="17" t="n"/>
-      <c r="H8" s="20">
-        <f>MAX(0,MIN(DATE(2025,12,31),IF(G8&gt;0,G8,DATE(2025,12,31)))-MAX(DATE(2025,1,1),IF(F8&gt;0,F8,DATE(2025,1,1)))+1)</f>
-        <v/>
-      </c>
-      <c r="I8" s="21">
+      <c r="D8" s="20" t="inlineStr"/>
+      <c r="E8" s="21" t="inlineStr"/>
+      <c r="F8" s="20" t="n"/>
+      <c r="G8" s="20" t="n"/>
+      <c r="H8" s="23">
+        <f>MAX(0,MIN(DATE(2025,12,31),IF(G8="",DATE(2025,12,31),G8))-MAX(DATE(2025,1,1),IF(F8="",DATE(2025,1,1),F8))+1)</f>
+        <v/>
+      </c>
+      <c r="I8" s="24">
         <f>H8/365</f>
         <v/>
       </c>
     </row>
+    <row r="9" ht="7.55" customHeight="1"/>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="26" t="inlineStr">
+        <is>
+          <t>Poste (lié au Récapitulatif)</t>
+        </is>
+      </c>
+      <c r="C10" s="27" t="inlineStr">
+        <is>
+          <t>Montant HT (€)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="15.05" customHeight="1">
+      <c r="A11" s="28">
+        <f>IFERROR(MID('Récapitulatif 2025'!A10,FIND(" — ",'Récapitulatif 2025'!A10)+4,100),"")</f>
+        <v/>
+      </c>
+      <c r="C11" s="29">
+        <f>'Récapitulatif 2025'!E10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="15.05" customHeight="1">
+      <c r="A12" s="28">
+        <f>IFERROR(MID('Récapitulatif 2025'!A21,FIND(" — ",'Récapitulatif 2025'!A21)+4,100),"")</f>
+        <v/>
+      </c>
+      <c r="C12" s="29">
+        <f>'Récapitulatif 2025'!E21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="15.05" customHeight="1">
+      <c r="A13" s="28">
+        <f>IFERROR(MID('Récapitulatif 2025'!A32,FIND(" — ",'Récapitulatif 2025'!A32)+4,100),"")</f>
+        <v/>
+      </c>
+      <c r="C13" s="29">
+        <f>'Récapitulatif 2025'!E32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="15.05" customHeight="1">
+      <c r="A14" s="28">
+        <f>IFERROR(MID('Récapitulatif 2025'!A37,FIND(" — ",'Récapitulatif 2025'!A37)+4,100),"")</f>
+        <v/>
+      </c>
+      <c r="C14" s="29">
+        <f>'Récapitulatif 2025'!E37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="15.05" customHeight="1">
+      <c r="A15" s="28">
+        <f>IFERROR(MID('Récapitulatif 2025'!A46,FIND(" — ",'Récapitulatif 2025'!A46)+4,100),"")</f>
+        <v/>
+      </c>
+      <c r="C15" s="29">
+        <f>'Récapitulatif 2025'!E46</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="15.05" customHeight="1">
+      <c r="A16" s="28">
+        <f>IFERROR(MID('Récapitulatif 2025'!A50,FIND(" — ",'Récapitulatif 2025'!A50)+4,100),"")</f>
+        <v/>
+      </c>
+      <c r="C16" s="29">
+        <f>'Récapitulatif 2025'!E50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="15.05" customHeight="1">
+      <c r="A17" s="28">
+        <f>IFERROR(MID('Récapitulatif 2025'!A54,FIND(" — ",'Récapitulatif 2025'!A54)+4,100),"")</f>
+        <v/>
+      </c>
+      <c r="C17" s="29">
+        <f>'Récapitulatif 2025'!E54</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="15.05" customHeight="1">
+      <c r="A18" s="28">
+        <f>IFERROR(MID('Récapitulatif 2025'!A59,FIND(" — ",'Récapitulatif 2025'!A59)+4,100),"")</f>
+        <v/>
+      </c>
+      <c r="C18" s="29">
+        <f>'Récapitulatif 2025'!E59</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="15.05" customHeight="1">
+      <c r="A19" s="28">
+        <f>IFERROR(MID('Récapitulatif 2025'!A64,FIND(" — ",'Récapitulatif 2025'!A64)+4,100),"")</f>
+        <v/>
+      </c>
+      <c r="C19" s="29">
+        <f>'Récapitulatif 2025'!E64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="15.05" customHeight="1">
+      <c r="A20" s="28">
+        <f>IFERROR(MID('Récapitulatif 2025'!A77,FIND(" — ",'Récapitulatif 2025'!A77)+4,100),"")</f>
+        <v/>
+      </c>
+      <c r="C20" s="29">
+        <f>'Récapitulatif 2025'!E77</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="15.05" customHeight="1">
+      <c r="A21" s="28">
+        <f>IFERROR(MID('Récapitulatif 2025'!A83,FIND(" — ",'Récapitulatif 2025'!A83)+4,100),"")</f>
+        <v/>
+      </c>
+      <c r="C21" s="29">
+        <f>'Récapitulatif 2025'!E83</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="15.05" customHeight="1">
+      <c r="A22" s="28">
+        <f>IFERROR(MID('Récapitulatif 2025'!A88,FIND(" — ",'Récapitulatif 2025'!A88)+4,100),"")</f>
+        <v/>
+      </c>
+      <c r="C22" s="29">
+        <f>'Récapitulatif 2025'!E88</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="15.05" customHeight="1">
+      <c r="A23" s="28">
+        <f>IFERROR(MID('Récapitulatif 2025'!A97,FIND(" — ",'Récapitulatif 2025'!A97)+4,100),"")</f>
+        <v/>
+      </c>
+      <c r="C23" s="29">
+        <f>'Récapitulatif 2025'!E97</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="15.05" customHeight="1">
+      <c r="A24" s="28">
+        <f>IFERROR(MID('Récapitulatif 2025'!A101,FIND(" — ",'Récapitulatif 2025'!A101)+4,100),"")</f>
+        <v/>
+      </c>
+      <c r="C24" s="29">
+        <f>'Récapitulatif 2025'!E101</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="15.05" customHeight="1">
+      <c r="A25" s="28">
+        <f>IFERROR(MID('Récapitulatif 2025'!A104,FIND(" — ",'Récapitulatif 2025'!A104)+4,100),"")</f>
+        <v/>
+      </c>
+      <c r="C25" s="29">
+        <f>'Récapitulatif 2025'!E104</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="15.05" customHeight="1">
+      <c r="A26" s="28">
+        <f>IFERROR(MID('Récapitulatif 2025'!A107,FIND(" — ",'Récapitulatif 2025'!A107)+4,100),"")</f>
+        <v/>
+      </c>
+      <c r="C26" s="29">
+        <f>'Récapitulatif 2025'!E107</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" ht="15.05" customHeight="1">
+      <c r="A27" s="28">
+        <f>IFERROR(MID('Récapitulatif 2025'!A111,FIND(" — ",'Récapitulatif 2025'!A111)+4,100),"")</f>
+        <v/>
+      </c>
+      <c r="C27" s="29">
+        <f>'Récapitulatif 2025'!E111</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="15.05" customHeight="1">
+      <c r="A28" s="28">
+        <f>IFERROR(MID('Récapitulatif 2025'!A118,FIND(" — ",'Récapitulatif 2025'!A118)+4,100),"")</f>
+        <v/>
+      </c>
+      <c r="C28" s="29">
+        <f>'Récapitulatif 2025'!E118</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A10:B10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3474,7 +3708,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="25.55" customHeight="1">
-      <c r="A1" s="23" t="inlineStr">
+      <c r="A1" s="30" t="inlineStr">
         <is>
           <t>RÉGULARISATION DE CHARGES — C1 C2</t>
         </is>
@@ -3533,82 +3767,82 @@
       </c>
     </row>
     <row r="6" ht="15.05" customHeight="1">
-      <c r="A6" s="24" t="inlineStr">
+      <c r="A6" s="31" t="inlineStr">
         <is>
           <t>Eau</t>
         </is>
       </c>
-      <c r="B6" s="25">
+      <c r="B6" s="32">
         <f>Paramètres!$C$7/Paramètres!$C$3</f>
         <v/>
       </c>
-      <c r="C6" s="26">
+      <c r="C6" s="33">
         <f>'Récapitulatif 2025'!E10</f>
         <v/>
       </c>
-      <c r="D6" s="26">
+      <c r="D6" s="33">
         <f>B6*C6</f>
         <v/>
       </c>
-      <c r="E6" s="27">
+      <c r="E6" s="34">
         <f>Paramètres!$H$7/365</f>
         <v/>
       </c>
-      <c r="F6" s="26">
+      <c r="F6" s="33">
         <f>D6*E6</f>
         <v/>
       </c>
     </row>
     <row r="7" ht="15.05" customHeight="1">
-      <c r="A7" s="24" t="inlineStr">
+      <c r="A7" s="31" t="inlineStr">
         <is>
           <t>Electricité</t>
         </is>
       </c>
-      <c r="B7" s="25">
+      <c r="B7" s="32">
         <f>Paramètres!$C$7/Paramètres!$C$3</f>
         <v/>
       </c>
-      <c r="C7" s="26">
+      <c r="C7" s="33">
         <f>'Récapitulatif 2025'!E21</f>
         <v/>
       </c>
-      <c r="D7" s="26">
+      <c r="D7" s="33">
         <f>B7*C7</f>
         <v/>
       </c>
-      <c r="E7" s="27">
+      <c r="E7" s="34">
         <f>Paramètres!$H$7/365</f>
         <v/>
       </c>
-      <c r="F7" s="26">
+      <c r="F7" s="33">
         <f>D7*E7</f>
         <v/>
       </c>
     </row>
     <row r="8" ht="15.05" customHeight="1">
-      <c r="A8" s="24" t="inlineStr">
+      <c r="A8" s="31" t="inlineStr">
         <is>
           <t>Gaz</t>
         </is>
       </c>
-      <c r="B8" s="25">
+      <c r="B8" s="32">
         <f>Paramètres!$C$7/Paramètres!$C$3</f>
         <v/>
       </c>
-      <c r="C8" s="26">
+      <c r="C8" s="33">
         <f>'Récapitulatif 2025'!E32</f>
         <v/>
       </c>
-      <c r="D8" s="26">
+      <c r="D8" s="33">
         <f>B8*C8</f>
         <v/>
       </c>
-      <c r="E8" s="27">
+      <c r="E8" s="34">
         <f>Paramètres!$H$7/365</f>
         <v/>
       </c>
-      <c r="F8" s="26">
+      <c r="F8" s="33">
         <f>D8*E8</f>
         <v/>
       </c>
@@ -3627,7 +3861,7 @@
         <f>SUM(D6:D8)</f>
         <v/>
       </c>
-      <c r="E9" s="28" t="n"/>
+      <c r="E9" s="35" t="n"/>
       <c r="F9" s="11">
         <f>SUM(F6:F8)</f>
         <v/>
@@ -3641,28 +3875,28 @@
       </c>
     </row>
     <row r="11" ht="15.05" customHeight="1">
-      <c r="A11" s="24" t="inlineStr">
+      <c r="A11" s="31" t="inlineStr">
         <is>
           <t>Entretien Courant</t>
         </is>
       </c>
-      <c r="B11" s="25">
+      <c r="B11" s="32">
         <f>Paramètres!$C$7/Paramètres!$C$3</f>
         <v/>
       </c>
-      <c r="C11" s="26">
+      <c r="C11" s="33">
         <f>'Récapitulatif 2025'!E37</f>
         <v/>
       </c>
-      <c r="D11" s="26">
+      <c r="D11" s="33">
         <f>B11*C11</f>
         <v/>
       </c>
-      <c r="E11" s="27">
+      <c r="E11" s="34">
         <f>Paramètres!$H$7/365</f>
         <v/>
       </c>
-      <c r="F11" s="26">
+      <c r="F11" s="33">
         <f>D11*E11</f>
         <v/>
       </c>
@@ -3681,7 +3915,7 @@
         <f>SUM(D11:D11)</f>
         <v/>
       </c>
-      <c r="E12" s="28" t="n"/>
+      <c r="E12" s="35" t="n"/>
       <c r="F12" s="11">
         <f>SUM(F11:F11)</f>
         <v/>
@@ -3695,325 +3929,325 @@
       </c>
     </row>
     <row r="14" ht="15.05" customHeight="1">
-      <c r="A14" s="24" t="inlineStr">
+      <c r="A14" s="31" t="inlineStr">
         <is>
           <t>Espaces Verts</t>
         </is>
       </c>
-      <c r="B14" s="25">
+      <c r="B14" s="32">
         <f>Paramètres!$C$7/Paramètres!$C$3</f>
         <v/>
       </c>
-      <c r="C14" s="26">
+      <c r="C14" s="33">
         <f>'Récapitulatif 2025'!E46</f>
         <v/>
       </c>
-      <c r="D14" s="26">
+      <c r="D14" s="33">
         <f>B14*C14</f>
         <v/>
       </c>
-      <c r="E14" s="27">
+      <c r="E14" s="34">
         <f>Paramètres!$H$7/365</f>
         <v/>
       </c>
-      <c r="F14" s="26">
+      <c r="F14" s="33">
         <f>D14*E14</f>
         <v/>
       </c>
     </row>
     <row r="15" ht="15.05" customHeight="1">
-      <c r="A15" s="24" t="inlineStr">
+      <c r="A15" s="31" t="inlineStr">
         <is>
           <t>CVC</t>
         </is>
       </c>
-      <c r="B15" s="25">
+      <c r="B15" s="32">
         <f>Paramètres!$C$7/Paramètres!$C$3</f>
         <v/>
       </c>
-      <c r="C15" s="26">
+      <c r="C15" s="33">
         <f>'Récapitulatif 2025'!E50</f>
         <v/>
       </c>
-      <c r="D15" s="26">
+      <c r="D15" s="33">
         <f>B15*C15</f>
         <v/>
       </c>
-      <c r="E15" s="27">
+      <c r="E15" s="34">
         <f>Paramètres!$H$7/365</f>
         <v/>
       </c>
-      <c r="F15" s="26">
+      <c r="F15" s="33">
         <f>D15*E15</f>
         <v/>
       </c>
     </row>
     <row r="16" ht="15.05" customHeight="1">
-      <c r="A16" s="24" t="inlineStr">
+      <c r="A16" s="31" t="inlineStr">
         <is>
           <t>Sécurité</t>
         </is>
       </c>
-      <c r="B16" s="25">
+      <c r="B16" s="32">
         <f>Paramètres!$C$7/Paramètres!$C$3</f>
         <v/>
       </c>
-      <c r="C16" s="26">
+      <c r="C16" s="33">
         <f>'Récapitulatif 2025'!E54</f>
         <v/>
       </c>
-      <c r="D16" s="26">
+      <c r="D16" s="33">
         <f>B16*C16</f>
         <v/>
       </c>
-      <c r="E16" s="27">
+      <c r="E16" s="34">
         <f>Paramètres!$H$7/365</f>
         <v/>
       </c>
-      <c r="F16" s="26">
+      <c r="F16" s="33">
         <f>D16*E16</f>
         <v/>
       </c>
     </row>
     <row r="17" ht="15.05" customHeight="1">
-      <c r="A17" s="24" t="inlineStr">
+      <c r="A17" s="31" t="inlineStr">
         <is>
           <t>SSI</t>
         </is>
       </c>
-      <c r="B17" s="25">
+      <c r="B17" s="32">
         <f>Paramètres!$C$7/Paramètres!$C$3</f>
         <v/>
       </c>
-      <c r="C17" s="26">
+      <c r="C17" s="33">
         <f>'Récapitulatif 2025'!E59</f>
         <v/>
       </c>
-      <c r="D17" s="26">
+      <c r="D17" s="33">
         <f>B17*C17</f>
         <v/>
       </c>
-      <c r="E17" s="27">
+      <c r="E17" s="34">
         <f>Paramètres!$H$7/365</f>
         <v/>
       </c>
-      <c r="F17" s="26">
+      <c r="F17" s="33">
         <f>D17*E17</f>
         <v/>
       </c>
     </row>
     <row r="18" ht="15.05" customHeight="1">
-      <c r="A18" s="24" t="inlineStr">
+      <c r="A18" s="31" t="inlineStr">
         <is>
           <t>Toitures</t>
         </is>
       </c>
-      <c r="B18" s="25">
+      <c r="B18" s="32">
         <f>Paramètres!$C$7/Paramètres!$C$3</f>
         <v/>
       </c>
-      <c r="C18" s="26">
+      <c r="C18" s="33">
         <f>'Récapitulatif 2025'!E64</f>
         <v/>
       </c>
-      <c r="D18" s="26">
+      <c r="D18" s="33">
         <f>B18*C18</f>
         <v/>
       </c>
-      <c r="E18" s="27">
+      <c r="E18" s="34">
         <f>Paramètres!$H$7/365</f>
         <v/>
       </c>
-      <c r="F18" s="26">
+      <c r="F18" s="33">
         <f>D18*E18</f>
         <v/>
       </c>
     </row>
     <row r="19" ht="15.05" customHeight="1">
-      <c r="A19" s="24" t="inlineStr">
+      <c r="A19" s="31" t="inlineStr">
         <is>
           <t>SPK / RIA / PI</t>
         </is>
       </c>
-      <c r="B19" s="25">
+      <c r="B19" s="32">
         <f>Paramètres!$C$7/Paramètres!$C$3</f>
         <v/>
       </c>
-      <c r="C19" s="26">
+      <c r="C19" s="33">
         <f>'Récapitulatif 2025'!E77</f>
         <v/>
       </c>
-      <c r="D19" s="26">
+      <c r="D19" s="33">
         <f>B19*C19</f>
         <v/>
       </c>
-      <c r="E19" s="27">
+      <c r="E19" s="34">
         <f>Paramètres!$H$7/365</f>
         <v/>
       </c>
-      <c r="F19" s="26">
+      <c r="F19" s="33">
         <f>D19*E19</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="15.05" customHeight="1">
-      <c r="A20" s="24" t="inlineStr">
+      <c r="A20" s="31" t="inlineStr">
         <is>
           <t>Installations électriques</t>
         </is>
       </c>
-      <c r="B20" s="25">
+      <c r="B20" s="32">
         <f>Paramètres!$C$7/35730.0</f>
         <v/>
       </c>
-      <c r="C20" s="26">
+      <c r="C20" s="33">
         <f>'Récapitulatif 2025'!E83</f>
         <v/>
       </c>
-      <c r="D20" s="26">
+      <c r="D20" s="33">
         <f>B20*C20</f>
         <v/>
       </c>
-      <c r="E20" s="27">
+      <c r="E20" s="34">
         <f>Paramètres!$H$7/365</f>
         <v/>
       </c>
-      <c r="F20" s="26">
+      <c r="F20" s="33">
         <f>D20*E20</f>
         <v/>
       </c>
     </row>
     <row r="21" ht="15.05" customHeight="1">
-      <c r="A21" s="24" t="inlineStr">
+      <c r="A21" s="31" t="inlineStr">
         <is>
           <t>Protection Foudre</t>
         </is>
       </c>
-      <c r="B21" s="25">
+      <c r="B21" s="32">
         <f>Paramètres!$C$7/23820.0</f>
         <v/>
       </c>
-      <c r="C21" s="26">
+      <c r="C21" s="33">
         <f>'Récapitulatif 2025'!E88</f>
         <v/>
       </c>
-      <c r="D21" s="26">
+      <c r="D21" s="33">
         <f>B21*C21</f>
         <v/>
       </c>
-      <c r="E21" s="27">
+      <c r="E21" s="34">
         <f>Paramètres!$H$7/365</f>
         <v/>
       </c>
-      <c r="F21" s="26">
+      <c r="F21" s="33">
         <f>D21*E21</f>
         <v/>
       </c>
     </row>
     <row r="22" ht="15.05" customHeight="1">
-      <c r="A22" s="24" t="inlineStr">
+      <c r="A22" s="31" t="inlineStr">
         <is>
           <t>GTB</t>
         </is>
       </c>
-      <c r="B22" s="25">
+      <c r="B22" s="32">
         <f>Paramètres!$C$7/Paramètres!$C$3</f>
         <v/>
       </c>
-      <c r="C22" s="26">
+      <c r="C22" s="33">
         <f>'Récapitulatif 2025'!E97</f>
         <v/>
       </c>
-      <c r="D22" s="26">
+      <c r="D22" s="33">
         <f>B22*C22</f>
         <v/>
       </c>
-      <c r="E22" s="27">
+      <c r="E22" s="34">
         <f>Paramètres!$H$7/365</f>
         <v/>
       </c>
-      <c r="F22" s="26">
+      <c r="F22" s="33">
         <f>D22*E22</f>
         <v/>
       </c>
     </row>
     <row r="23" ht="15.05" customHeight="1">
-      <c r="A23" s="24" t="inlineStr">
+      <c r="A23" s="31" t="inlineStr">
         <is>
           <t>Détection Gaz</t>
         </is>
       </c>
-      <c r="B23" s="25">
+      <c r="B23" s="32">
         <f>Paramètres!$C$7/Paramètres!$C$3</f>
         <v/>
       </c>
-      <c r="C23" s="26">
+      <c r="C23" s="33">
         <f>'Récapitulatif 2025'!E101</f>
         <v/>
       </c>
-      <c r="D23" s="26">
+      <c r="D23" s="33">
         <f>B23*C23</f>
         <v/>
       </c>
-      <c r="E23" s="27">
+      <c r="E23" s="34">
         <f>Paramètres!$H$7/365</f>
         <v/>
       </c>
-      <c r="F23" s="26">
+      <c r="F23" s="33">
         <f>D23*E23</f>
         <v/>
       </c>
     </row>
     <row r="24" ht="15.05" customHeight="1">
-      <c r="A24" s="24" t="inlineStr">
+      <c r="A24" s="31" t="inlineStr">
         <is>
           <t>Vérifications règlementaires</t>
         </is>
       </c>
-      <c r="B24" s="25">
+      <c r="B24" s="32">
         <f>Paramètres!$C$7/19945.0</f>
         <v/>
       </c>
-      <c r="C24" s="26">
+      <c r="C24" s="33">
         <f>'Récapitulatif 2025'!E104</f>
         <v/>
       </c>
-      <c r="D24" s="26">
+      <c r="D24" s="33">
         <f>B24*C24</f>
         <v/>
       </c>
-      <c r="E24" s="27">
+      <c r="E24" s="34">
         <f>Paramètres!$H$7/365</f>
         <v/>
       </c>
-      <c r="F24" s="26">
+      <c r="F24" s="33">
         <f>D24*E24</f>
         <v/>
       </c>
     </row>
     <row r="25" ht="15.05" customHeight="1">
-      <c r="A25" s="24" t="inlineStr">
+      <c r="A25" s="31" t="inlineStr">
         <is>
           <t>Portails</t>
         </is>
       </c>
-      <c r="B25" s="25">
+      <c r="B25" s="32">
         <f>Paramètres!$C$7/Paramètres!$C$3</f>
         <v/>
       </c>
-      <c r="C25" s="26">
+      <c r="C25" s="33">
         <f>'Récapitulatif 2025'!E107</f>
         <v/>
       </c>
-      <c r="D25" s="26">
+      <c r="D25" s="33">
         <f>B25*C25</f>
         <v/>
       </c>
-      <c r="E25" s="27">
+      <c r="E25" s="34">
         <f>Paramètres!$H$7/365</f>
         <v/>
       </c>
-      <c r="F25" s="26">
+      <c r="F25" s="33">
         <f>D25*E25</f>
         <v/>
       </c>
@@ -4032,7 +4266,7 @@
         <f>SUM(D14:D25)</f>
         <v/>
       </c>
-      <c r="E26" s="28" t="n"/>
+      <c r="E26" s="35" t="n"/>
       <c r="F26" s="11">
         <f>SUM(F14:F25)</f>
         <v/>
@@ -4046,28 +4280,28 @@
       </c>
     </row>
     <row r="28" ht="15.05" customHeight="1">
-      <c r="A28" s="24" t="inlineStr">
+      <c r="A28" s="31" t="inlineStr">
         <is>
           <t>Assurances</t>
         </is>
       </c>
-      <c r="B28" s="25">
+      <c r="B28" s="32">
         <f>Paramètres!$C$7/Paramètres!$C$3</f>
         <v/>
       </c>
-      <c r="C28" s="26">
+      <c r="C28" s="33">
         <f>'Récapitulatif 2025'!E111</f>
         <v/>
       </c>
-      <c r="D28" s="26">
+      <c r="D28" s="33">
         <f>B28*C28</f>
         <v/>
       </c>
-      <c r="E28" s="27">
+      <c r="E28" s="34">
         <f>Paramètres!$H$7/365</f>
         <v/>
       </c>
-      <c r="F28" s="26">
+      <c r="F28" s="33">
         <f>D28*E28</f>
         <v/>
       </c>
@@ -4086,7 +4320,7 @@
         <f>SUM(D28:D28)</f>
         <v/>
       </c>
-      <c r="E29" s="28" t="n"/>
+      <c r="E29" s="35" t="n"/>
       <c r="F29" s="11">
         <f>SUM(F28:F28)</f>
         <v/>
@@ -4094,21 +4328,21 @@
     </row>
     <row r="30" ht="7.55" customHeight="1"/>
     <row r="31" ht="21.75" customHeight="1">
-      <c r="A31" s="29" t="inlineStr">
+      <c r="A31" s="15" t="inlineStr">
         <is>
           <t>TOTAL CHARGES RÉCUPÉRABLES RÉELLES (€ HT)</t>
         </is>
       </c>
-      <c r="C31" s="30">
+      <c r="C31" s="16">
         <f>C9+C12+C26+C29</f>
         <v/>
       </c>
-      <c r="D31" s="30">
+      <c r="D31" s="16">
         <f>D9+D12+D26+D29</f>
         <v/>
       </c>
-      <c r="E31" s="31" t="n"/>
-      <c r="F31" s="30">
+      <c r="E31" s="36" t="n"/>
+      <c r="F31" s="16">
         <f>F9+F12+F26+F29</f>
         <v/>
       </c>
@@ -4120,56 +4354,56 @@
           <t>Provisions pour charges versées</t>
         </is>
       </c>
-      <c r="C33" s="32" t="n"/>
-      <c r="D33" s="33" t="inlineStr">
+      <c r="C33" s="37" t="n"/>
+      <c r="D33" s="27" t="inlineStr">
         <is>
           <t>Montant annuel (€)</t>
         </is>
       </c>
-      <c r="E33" s="32" t="n"/>
-      <c r="F33" s="33" t="inlineStr">
+      <c r="E33" s="37" t="n"/>
+      <c r="F33" s="27" t="inlineStr">
         <is>
           <t>Montant locataire (€)</t>
         </is>
       </c>
     </row>
     <row r="34" ht="15.8" customHeight="1">
-      <c r="A34" s="18" t="inlineStr">
+      <c r="A34" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">  1er trimestre (T1)</t>
         </is>
       </c>
-      <c r="F34" s="26" t="n">
+      <c r="F34" s="33" t="n">
         <v>2990.6</v>
       </c>
     </row>
     <row r="35" ht="15.8" customHeight="1">
-      <c r="A35" s="18" t="inlineStr">
+      <c r="A35" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">  2e trimestre (T2)</t>
         </is>
       </c>
-      <c r="F35" s="26" t="n">
+      <c r="F35" s="33" t="n">
         <v>25284.11</v>
       </c>
     </row>
     <row r="36" ht="15.8" customHeight="1">
-      <c r="A36" s="18" t="inlineStr">
+      <c r="A36" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">  3e trimestre (T3)</t>
         </is>
       </c>
-      <c r="F36" s="26" t="n">
+      <c r="F36" s="33" t="n">
         <v>28376.42</v>
       </c>
     </row>
     <row r="37" ht="15.8" customHeight="1">
-      <c r="A37" s="18" t="inlineStr">
+      <c r="A37" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">  4e trimestre (T4)</t>
         </is>
       </c>
-      <c r="F37" s="26" t="n">
+      <c r="F37" s="33" t="n">
         <v>28376.42</v>
       </c>
     </row>
@@ -4183,7 +4417,7 @@
         <f>SUM(D34:D37)</f>
         <v/>
       </c>
-      <c r="E38" s="28" t="n"/>
+      <c r="E38" s="35" t="n"/>
       <c r="F38" s="11">
         <f>SUM(F34:F37)</f>
         <v/>
@@ -4191,22 +4425,22 @@
     </row>
     <row r="39" ht="7.55" customHeight="1"/>
     <row r="40" ht="21.75" customHeight="1">
-      <c r="A40" s="34">
+      <c r="A40" s="38">
         <f>IF(F31-F38&gt;0,"SOLDE DÉBITEUR","SOLDE CRÉDITEUR")</f>
         <v/>
       </c>
-      <c r="D40" s="35">
+      <c r="D40" s="39">
         <f>D31-D38</f>
         <v/>
       </c>
-      <c r="E40" s="32" t="n"/>
-      <c r="F40" s="35">
+      <c r="E40" s="37" t="n"/>
+      <c r="F40" s="39">
         <f>F31-F38</f>
         <v/>
       </c>
     </row>
     <row r="42" ht="27.75" customHeight="1">
-      <c r="A42" s="36" t="inlineStr">
+      <c r="A42" s="40" t="inlineStr">
         <is>
           <t>ℹ  Clé répartition = surface lot ÷ surface totale site. Période = nombre de jours d'occupation ÷ 365.</t>
         </is>
@@ -4252,7 +4486,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="25.55" customHeight="1">
-      <c r="A1" s="23" t="inlineStr">
+      <c r="A1" s="30" t="inlineStr">
         <is>
           <t>RÉGULARISATION DE CHARGES — C3 C4 C5</t>
         </is>
@@ -4311,82 +4545,82 @@
       </c>
     </row>
     <row r="6" ht="15.05" customHeight="1">
-      <c r="A6" s="24" t="inlineStr">
+      <c r="A6" s="31" t="inlineStr">
         <is>
           <t>Eau</t>
         </is>
       </c>
-      <c r="B6" s="25">
+      <c r="B6" s="32">
         <f>Paramètres!$C$8/Paramètres!$C$3</f>
         <v/>
       </c>
-      <c r="C6" s="26">
+      <c r="C6" s="33">
         <f>'Récapitulatif 2025'!E10</f>
         <v/>
       </c>
-      <c r="D6" s="26">
+      <c r="D6" s="33">
         <f>B6*C6</f>
         <v/>
       </c>
-      <c r="E6" s="27">
+      <c r="E6" s="34">
         <f>Paramètres!$H$8/365</f>
         <v/>
       </c>
-      <c r="F6" s="26">
+      <c r="F6" s="33">
         <f>D6*E6</f>
         <v/>
       </c>
     </row>
     <row r="7" ht="15.05" customHeight="1">
-      <c r="A7" s="24" t="inlineStr">
+      <c r="A7" s="31" t="inlineStr">
         <is>
           <t>Electricité</t>
         </is>
       </c>
-      <c r="B7" s="25">
+      <c r="B7" s="32">
         <f>Paramètres!$C$8/Paramètres!$C$3</f>
         <v/>
       </c>
-      <c r="C7" s="26">
+      <c r="C7" s="33">
         <f>'Récapitulatif 2025'!E21</f>
         <v/>
       </c>
-      <c r="D7" s="26">
+      <c r="D7" s="33">
         <f>B7*C7</f>
         <v/>
       </c>
-      <c r="E7" s="27">
+      <c r="E7" s="34">
         <f>Paramètres!$H$8/365</f>
         <v/>
       </c>
-      <c r="F7" s="26">
+      <c r="F7" s="33">
         <f>D7*E7</f>
         <v/>
       </c>
     </row>
     <row r="8" ht="15.05" customHeight="1">
-      <c r="A8" s="24" t="inlineStr">
+      <c r="A8" s="31" t="inlineStr">
         <is>
           <t>Gaz</t>
         </is>
       </c>
-      <c r="B8" s="25">
+      <c r="B8" s="32">
         <f>Paramètres!$C$8/Paramètres!$C$3</f>
         <v/>
       </c>
-      <c r="C8" s="26">
+      <c r="C8" s="33">
         <f>'Récapitulatif 2025'!E32</f>
         <v/>
       </c>
-      <c r="D8" s="26">
+      <c r="D8" s="33">
         <f>B8*C8</f>
         <v/>
       </c>
-      <c r="E8" s="27">
+      <c r="E8" s="34">
         <f>Paramètres!$H$8/365</f>
         <v/>
       </c>
-      <c r="F8" s="26">
+      <c r="F8" s="33">
         <f>D8*E8</f>
         <v/>
       </c>
@@ -4405,7 +4639,7 @@
         <f>SUM(D6:D8)</f>
         <v/>
       </c>
-      <c r="E9" s="28" t="n"/>
+      <c r="E9" s="35" t="n"/>
       <c r="F9" s="11">
         <f>SUM(F6:F8)</f>
         <v/>
@@ -4419,28 +4653,28 @@
       </c>
     </row>
     <row r="11" ht="15.05" customHeight="1">
-      <c r="A11" s="24" t="inlineStr">
+      <c r="A11" s="31" t="inlineStr">
         <is>
           <t>Entretien Courant</t>
         </is>
       </c>
-      <c r="B11" s="25">
+      <c r="B11" s="32">
         <f>Paramètres!$C$8/Paramètres!$C$3</f>
         <v/>
       </c>
-      <c r="C11" s="26">
+      <c r="C11" s="33">
         <f>'Récapitulatif 2025'!E37</f>
         <v/>
       </c>
-      <c r="D11" s="26">
+      <c r="D11" s="33">
         <f>B11*C11</f>
         <v/>
       </c>
-      <c r="E11" s="27">
+      <c r="E11" s="34">
         <f>Paramètres!$H$8/365</f>
         <v/>
       </c>
-      <c r="F11" s="26">
+      <c r="F11" s="33">
         <f>D11*E11</f>
         <v/>
       </c>
@@ -4459,7 +4693,7 @@
         <f>SUM(D11:D11)</f>
         <v/>
       </c>
-      <c r="E12" s="28" t="n"/>
+      <c r="E12" s="35" t="n"/>
       <c r="F12" s="11">
         <f>SUM(F11:F11)</f>
         <v/>
@@ -4473,325 +4707,325 @@
       </c>
     </row>
     <row r="14" ht="15.05" customHeight="1">
-      <c r="A14" s="24" t="inlineStr">
+      <c r="A14" s="31" t="inlineStr">
         <is>
           <t>Espaces Verts</t>
         </is>
       </c>
-      <c r="B14" s="25">
+      <c r="B14" s="32">
         <f>Paramètres!$C$8/Paramètres!$C$3</f>
         <v/>
       </c>
-      <c r="C14" s="26">
+      <c r="C14" s="33">
         <f>'Récapitulatif 2025'!E46</f>
         <v/>
       </c>
-      <c r="D14" s="26">
+      <c r="D14" s="33">
         <f>B14*C14</f>
         <v/>
       </c>
-      <c r="E14" s="27">
+      <c r="E14" s="34">
         <f>Paramètres!$H$8/365</f>
         <v/>
       </c>
-      <c r="F14" s="26">
+      <c r="F14" s="33">
         <f>D14*E14</f>
         <v/>
       </c>
     </row>
     <row r="15" ht="15.05" customHeight="1">
-      <c r="A15" s="24" t="inlineStr">
+      <c r="A15" s="31" t="inlineStr">
         <is>
           <t>CVC</t>
         </is>
       </c>
-      <c r="B15" s="25">
+      <c r="B15" s="32">
         <f>Paramètres!$C$8/Paramètres!$C$3</f>
         <v/>
       </c>
-      <c r="C15" s="26">
+      <c r="C15" s="33">
         <f>'Récapitulatif 2025'!E50</f>
         <v/>
       </c>
-      <c r="D15" s="26">
+      <c r="D15" s="33">
         <f>B15*C15</f>
         <v/>
       </c>
-      <c r="E15" s="27">
+      <c r="E15" s="34">
         <f>Paramètres!$H$8/365</f>
         <v/>
       </c>
-      <c r="F15" s="26">
+      <c r="F15" s="33">
         <f>D15*E15</f>
         <v/>
       </c>
     </row>
     <row r="16" ht="15.05" customHeight="1">
-      <c r="A16" s="24" t="inlineStr">
+      <c r="A16" s="31" t="inlineStr">
         <is>
           <t>Sécurité</t>
         </is>
       </c>
-      <c r="B16" s="25">
+      <c r="B16" s="32">
         <f>Paramètres!$C$8/Paramètres!$C$3</f>
         <v/>
       </c>
-      <c r="C16" s="26">
+      <c r="C16" s="33">
         <f>'Récapitulatif 2025'!E54</f>
         <v/>
       </c>
-      <c r="D16" s="26">
+      <c r="D16" s="33">
         <f>B16*C16</f>
         <v/>
       </c>
-      <c r="E16" s="27">
+      <c r="E16" s="34">
         <f>Paramètres!$H$8/365</f>
         <v/>
       </c>
-      <c r="F16" s="26">
+      <c r="F16" s="33">
         <f>D16*E16</f>
         <v/>
       </c>
     </row>
     <row r="17" ht="15.05" customHeight="1">
-      <c r="A17" s="24" t="inlineStr">
+      <c r="A17" s="31" t="inlineStr">
         <is>
           <t>SSI</t>
         </is>
       </c>
-      <c r="B17" s="25">
+      <c r="B17" s="32">
         <f>Paramètres!$C$8/Paramètres!$C$3</f>
         <v/>
       </c>
-      <c r="C17" s="26">
+      <c r="C17" s="33">
         <f>'Récapitulatif 2025'!E59</f>
         <v/>
       </c>
-      <c r="D17" s="26">
+      <c r="D17" s="33">
         <f>B17*C17</f>
         <v/>
       </c>
-      <c r="E17" s="27">
+      <c r="E17" s="34">
         <f>Paramètres!$H$8/365</f>
         <v/>
       </c>
-      <c r="F17" s="26">
+      <c r="F17" s="33">
         <f>D17*E17</f>
         <v/>
       </c>
     </row>
     <row r="18" ht="15.05" customHeight="1">
-      <c r="A18" s="24" t="inlineStr">
+      <c r="A18" s="31" t="inlineStr">
         <is>
           <t>Toitures</t>
         </is>
       </c>
-      <c r="B18" s="25">
+      <c r="B18" s="32">
         <f>Paramètres!$C$8/Paramètres!$C$3</f>
         <v/>
       </c>
-      <c r="C18" s="26">
+      <c r="C18" s="33">
         <f>'Récapitulatif 2025'!E64</f>
         <v/>
       </c>
-      <c r="D18" s="26">
+      <c r="D18" s="33">
         <f>B18*C18</f>
         <v/>
       </c>
-      <c r="E18" s="27">
+      <c r="E18" s="34">
         <f>Paramètres!$H$8/365</f>
         <v/>
       </c>
-      <c r="F18" s="26">
+      <c r="F18" s="33">
         <f>D18*E18</f>
         <v/>
       </c>
     </row>
     <row r="19" ht="15.05" customHeight="1">
-      <c r="A19" s="24" t="inlineStr">
+      <c r="A19" s="31" t="inlineStr">
         <is>
           <t>SPK / RIA / PI</t>
         </is>
       </c>
-      <c r="B19" s="25">
+      <c r="B19" s="32">
         <f>Paramètres!$C$8/Paramètres!$C$3</f>
         <v/>
       </c>
-      <c r="C19" s="26">
+      <c r="C19" s="33">
         <f>'Récapitulatif 2025'!E77</f>
         <v/>
       </c>
-      <c r="D19" s="26">
+      <c r="D19" s="33">
         <f>B19*C19</f>
         <v/>
       </c>
-      <c r="E19" s="27">
+      <c r="E19" s="34">
         <f>Paramètres!$H$8/365</f>
         <v/>
       </c>
-      <c r="F19" s="26">
+      <c r="F19" s="33">
         <f>D19*E19</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="15.05" customHeight="1">
-      <c r="A20" s="24" t="inlineStr">
+      <c r="A20" s="31" t="inlineStr">
         <is>
           <t>Installations électriques</t>
         </is>
       </c>
-      <c r="B20" s="25">
+      <c r="B20" s="32">
         <f>Paramètres!$C$8/35730.0</f>
         <v/>
       </c>
-      <c r="C20" s="26">
+      <c r="C20" s="33">
         <f>'Récapitulatif 2025'!E83</f>
         <v/>
       </c>
-      <c r="D20" s="26">
+      <c r="D20" s="33">
         <f>B20*C20</f>
         <v/>
       </c>
-      <c r="E20" s="27">
+      <c r="E20" s="34">
         <f>Paramètres!$H$8/365</f>
         <v/>
       </c>
-      <c r="F20" s="26">
+      <c r="F20" s="33">
         <f>D20*E20</f>
         <v/>
       </c>
     </row>
     <row r="21" ht="15.05" customHeight="1">
-      <c r="A21" s="24" t="inlineStr">
+      <c r="A21" s="31" t="inlineStr">
         <is>
           <t>Protection Foudre</t>
         </is>
       </c>
-      <c r="B21" s="25">
+      <c r="B21" s="32">
         <f>Paramètres!$C$8/23820.0</f>
         <v/>
       </c>
-      <c r="C21" s="26">
+      <c r="C21" s="33">
         <f>'Récapitulatif 2025'!E88</f>
         <v/>
       </c>
-      <c r="D21" s="26">
+      <c r="D21" s="33">
         <f>B21*C21</f>
         <v/>
       </c>
-      <c r="E21" s="27">
+      <c r="E21" s="34">
         <f>Paramètres!$H$8/365</f>
         <v/>
       </c>
-      <c r="F21" s="26">
+      <c r="F21" s="33">
         <f>D21*E21</f>
         <v/>
       </c>
     </row>
     <row r="22" ht="15.05" customHeight="1">
-      <c r="A22" s="24" t="inlineStr">
+      <c r="A22" s="31" t="inlineStr">
         <is>
           <t>GTB</t>
         </is>
       </c>
-      <c r="B22" s="25">
+      <c r="B22" s="32">
         <f>Paramètres!$C$8/Paramètres!$C$3</f>
         <v/>
       </c>
-      <c r="C22" s="26">
+      <c r="C22" s="33">
         <f>'Récapitulatif 2025'!E97</f>
         <v/>
       </c>
-      <c r="D22" s="26">
+      <c r="D22" s="33">
         <f>B22*C22</f>
         <v/>
       </c>
-      <c r="E22" s="27">
+      <c r="E22" s="34">
         <f>Paramètres!$H$8/365</f>
         <v/>
       </c>
-      <c r="F22" s="26">
+      <c r="F22" s="33">
         <f>D22*E22</f>
         <v/>
       </c>
     </row>
     <row r="23" ht="15.05" customHeight="1">
-      <c r="A23" s="24" t="inlineStr">
+      <c r="A23" s="31" t="inlineStr">
         <is>
           <t>Détection Gaz</t>
         </is>
       </c>
-      <c r="B23" s="25">
+      <c r="B23" s="32">
         <f>Paramètres!$C$8/Paramètres!$C$3</f>
         <v/>
       </c>
-      <c r="C23" s="26">
+      <c r="C23" s="33">
         <f>'Récapitulatif 2025'!E101</f>
         <v/>
       </c>
-      <c r="D23" s="26">
+      <c r="D23" s="33">
         <f>B23*C23</f>
         <v/>
       </c>
-      <c r="E23" s="27">
+      <c r="E23" s="34">
         <f>Paramètres!$H$8/365</f>
         <v/>
       </c>
-      <c r="F23" s="26">
+      <c r="F23" s="33">
         <f>D23*E23</f>
         <v/>
       </c>
     </row>
     <row r="24" ht="15.05" customHeight="1">
-      <c r="A24" s="24" t="inlineStr">
+      <c r="A24" s="31" t="inlineStr">
         <is>
           <t>Vérifications règlementaires</t>
         </is>
       </c>
-      <c r="B24" s="25">
+      <c r="B24" s="32">
         <f>Paramètres!$C$8/19945.0</f>
         <v/>
       </c>
-      <c r="C24" s="26">
+      <c r="C24" s="33">
         <f>'Récapitulatif 2025'!E104</f>
         <v/>
       </c>
-      <c r="D24" s="26">
+      <c r="D24" s="33">
         <f>B24*C24</f>
         <v/>
       </c>
-      <c r="E24" s="27">
+      <c r="E24" s="34">
         <f>Paramètres!$H$8/365</f>
         <v/>
       </c>
-      <c r="F24" s="26">
+      <c r="F24" s="33">
         <f>D24*E24</f>
         <v/>
       </c>
     </row>
     <row r="25" ht="15.05" customHeight="1">
-      <c r="A25" s="24" t="inlineStr">
+      <c r="A25" s="31" t="inlineStr">
         <is>
           <t>Portails</t>
         </is>
       </c>
-      <c r="B25" s="25">
+      <c r="B25" s="32">
         <f>Paramètres!$C$8/Paramètres!$C$3</f>
         <v/>
       </c>
-      <c r="C25" s="26">
+      <c r="C25" s="33">
         <f>'Récapitulatif 2025'!E107</f>
         <v/>
       </c>
-      <c r="D25" s="26">
+      <c r="D25" s="33">
         <f>B25*C25</f>
         <v/>
       </c>
-      <c r="E25" s="27">
+      <c r="E25" s="34">
         <f>Paramètres!$H$8/365</f>
         <v/>
       </c>
-      <c r="F25" s="26">
+      <c r="F25" s="33">
         <f>D25*E25</f>
         <v/>
       </c>
@@ -4810,7 +5044,7 @@
         <f>SUM(D14:D25)</f>
         <v/>
       </c>
-      <c r="E26" s="28" t="n"/>
+      <c r="E26" s="35" t="n"/>
       <c r="F26" s="11">
         <f>SUM(F14:F25)</f>
         <v/>
@@ -4824,28 +5058,28 @@
       </c>
     </row>
     <row r="28" ht="15.05" customHeight="1">
-      <c r="A28" s="24" t="inlineStr">
+      <c r="A28" s="31" t="inlineStr">
         <is>
           <t>Assurances</t>
         </is>
       </c>
-      <c r="B28" s="25">
+      <c r="B28" s="32">
         <f>Paramètres!$C$8/Paramètres!$C$3</f>
         <v/>
       </c>
-      <c r="C28" s="26">
+      <c r="C28" s="33">
         <f>'Récapitulatif 2025'!E111</f>
         <v/>
       </c>
-      <c r="D28" s="26">
+      <c r="D28" s="33">
         <f>B28*C28</f>
         <v/>
       </c>
-      <c r="E28" s="27">
+      <c r="E28" s="34">
         <f>Paramètres!$H$8/365</f>
         <v/>
       </c>
-      <c r="F28" s="26">
+      <c r="F28" s="33">
         <f>D28*E28</f>
         <v/>
       </c>
@@ -4864,7 +5098,7 @@
         <f>SUM(D28:D28)</f>
         <v/>
       </c>
-      <c r="E29" s="28" t="n"/>
+      <c r="E29" s="35" t="n"/>
       <c r="F29" s="11">
         <f>SUM(F28:F28)</f>
         <v/>
@@ -4872,21 +5106,21 @@
     </row>
     <row r="30" ht="7.55" customHeight="1"/>
     <row r="31" ht="21.75" customHeight="1">
-      <c r="A31" s="29" t="inlineStr">
+      <c r="A31" s="15" t="inlineStr">
         <is>
           <t>TOTAL CHARGES RÉCUPÉRABLES RÉELLES (€ HT)</t>
         </is>
       </c>
-      <c r="C31" s="30">
+      <c r="C31" s="16">
         <f>C9+C12+C26+C29</f>
         <v/>
       </c>
-      <c r="D31" s="30">
+      <c r="D31" s="16">
         <f>D9+D12+D26+D29</f>
         <v/>
       </c>
-      <c r="E31" s="31" t="n"/>
-      <c r="F31" s="30">
+      <c r="E31" s="36" t="n"/>
+      <c r="F31" s="16">
         <f>F9+F12+F26+F29</f>
         <v/>
       </c>
@@ -4898,42 +5132,42 @@
           <t>Provisions pour charges versées</t>
         </is>
       </c>
-      <c r="C33" s="32" t="n"/>
-      <c r="D33" s="33" t="inlineStr">
+      <c r="C33" s="37" t="n"/>
+      <c r="D33" s="27" t="inlineStr">
         <is>
           <t>Montant annuel (€)</t>
         </is>
       </c>
-      <c r="E33" s="32" t="n"/>
-      <c r="F33" s="33" t="inlineStr">
+      <c r="E33" s="37" t="n"/>
+      <c r="F33" s="27" t="inlineStr">
         <is>
           <t>Montant locataire (€)</t>
         </is>
       </c>
     </row>
     <row r="34" ht="15.8" customHeight="1">
-      <c r="A34" s="18" t="inlineStr">
+      <c r="A34" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">  1er trimestre (T1)</t>
         </is>
       </c>
     </row>
     <row r="35" ht="15.8" customHeight="1">
-      <c r="A35" s="18" t="inlineStr">
+      <c r="A35" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">  2e trimestre (T2)</t>
         </is>
       </c>
     </row>
     <row r="36" ht="15.8" customHeight="1">
-      <c r="A36" s="18" t="inlineStr">
+      <c r="A36" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">  3e trimestre (T3)</t>
         </is>
       </c>
     </row>
     <row r="37" ht="15.8" customHeight="1">
-      <c r="A37" s="18" t="inlineStr">
+      <c r="A37" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">  4e trimestre (T4)</t>
         </is>
@@ -4949,7 +5183,7 @@
         <f>SUM(D34:D37)</f>
         <v/>
       </c>
-      <c r="E38" s="28" t="n"/>
+      <c r="E38" s="35" t="n"/>
       <c r="F38" s="11">
         <f>SUM(F34:F37)</f>
         <v/>
@@ -4957,22 +5191,22 @@
     </row>
     <row r="39" ht="7.55" customHeight="1"/>
     <row r="40" ht="21.75" customHeight="1">
-      <c r="A40" s="34">
+      <c r="A40" s="38">
         <f>IF(F31-F38&gt;0,"SOLDE DÉBITEUR","SOLDE CRÉDITEUR")</f>
         <v/>
       </c>
-      <c r="D40" s="35">
+      <c r="D40" s="39">
         <f>D31-D38</f>
         <v/>
       </c>
-      <c r="E40" s="32" t="n"/>
-      <c r="F40" s="35">
+      <c r="E40" s="37" t="n"/>
+      <c r="F40" s="39">
         <f>F31-F38</f>
         <v/>
       </c>
     </row>
     <row r="42" ht="27.75" customHeight="1">
-      <c r="A42" s="36" t="inlineStr">
+      <c r="A42" s="40" t="inlineStr">
         <is>
           <t>ℹ  Clé répartition = surface lot ÷ surface totale site. Période = nombre de jours d'occupation ÷ 365.</t>
         </is>
@@ -5019,7 +5253,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="25.55" customHeight="1">
-      <c r="A1" s="23" t="inlineStr">
+      <c r="A1" s="30" t="inlineStr">
         <is>
           <t>ORMES A — COÛT DE LA VACANCE LOCATIVE 2025</t>
         </is>
@@ -5066,54 +5300,54 @@
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="37">
+      <c r="A5" s="41">
         <f>Paramètres!A7</f>
         <v/>
       </c>
-      <c r="B5" s="17">
+      <c r="B5" s="20">
         <f>Paramètres!B7</f>
         <v/>
       </c>
-      <c r="C5" s="38">
+      <c r="C5" s="42">
         <f>Paramètres!C7</f>
         <v/>
       </c>
-      <c r="D5" s="26">
+      <c r="D5" s="33">
         <f>'C1 C2'!D31</f>
         <v/>
       </c>
-      <c r="E5" s="27">
+      <c r="E5" s="34">
         <f>Paramètres!H7/365</f>
         <v/>
       </c>
-      <c r="F5" s="39">
-        <f>IF(Paramètres!B7="Vacant",'C1 C2'!D31,'C1 C2'!D31*(1-Paramètres!H7/365))</f>
+      <c r="F5" s="29">
+        <f>IF(Paramètres!B7="Vacant",'C1 C2'!D31,'C1 C2'!D31-'C1 C2'!F31)</f>
         <v/>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="37">
+      <c r="A6" s="41">
         <f>Paramètres!A8</f>
         <v/>
       </c>
-      <c r="B6" s="17">
+      <c r="B6" s="20">
         <f>Paramètres!B8</f>
         <v/>
       </c>
-      <c r="C6" s="38">
+      <c r="C6" s="42">
         <f>Paramètres!C8</f>
         <v/>
       </c>
-      <c r="D6" s="26">
+      <c r="D6" s="33">
         <f>'C3 C4 C5'!D31</f>
         <v/>
       </c>
-      <c r="E6" s="27">
+      <c r="E6" s="34">
         <f>Paramètres!H8/365</f>
         <v/>
       </c>
-      <c r="F6" s="39">
-        <f>IF(Paramètres!B8="Vacant",'C3 C4 C5'!D31,'C3 C4 C5'!D31*(1-Paramètres!H8/365))</f>
+      <c r="F6" s="29">
+        <f>IF(Paramètres!B8="Vacant",'C3 C4 C5'!D31,'C3 C4 C5'!D31-'C3 C4 C5'!F31)</f>
         <v/>
       </c>
     </row>
@@ -5128,8 +5362,8 @@
         <f>SUM(D5:D6)</f>
         <v/>
       </c>
-      <c r="E8" s="28" t="n"/>
-      <c r="F8" s="28" t="n"/>
+      <c r="E8" s="35" t="n"/>
+      <c r="F8" s="35" t="n"/>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
@@ -5137,33 +5371,33 @@
           <t>Nombre de lots vacants</t>
         </is>
       </c>
-      <c r="D9" s="40">
+      <c r="D9" s="43">
         <f>COUNTIF(B5:B6,"Vacant")</f>
         <v/>
       </c>
-      <c r="E9" s="28" t="n"/>
-      <c r="F9" s="28" t="n"/>
+      <c r="E9" s="35" t="n"/>
+      <c r="F9" s="35" t="n"/>
     </row>
     <row r="10" ht="6" customHeight="1"/>
     <row r="11" ht="19.55" customHeight="1">
-      <c r="A11" s="41" t="inlineStr">
+      <c r="A11" s="44" t="inlineStr">
         <is>
           <t>Charges non récupérables (Frais Bancaires + CAPEX)</t>
         </is>
       </c>
-      <c r="F11" s="42">
+      <c r="F11" s="45">
         <f>'Récapitulatif 2025'!E118</f>
         <v/>
       </c>
     </row>
     <row r="12" ht="6" customHeight="1"/>
     <row r="13" ht="25.55" customHeight="1">
-      <c r="A13" s="43" t="inlineStr">
+      <c r="A13" s="46" t="inlineStr">
         <is>
           <t>TOTAL COÛT DE LA VACANCE LOCATIVE (€ HT)</t>
         </is>
       </c>
-      <c r="F13" s="44">
+      <c r="F13" s="47">
         <f>F5+F6+F11</f>
         <v/>
       </c>
@@ -5175,14 +5409,14 @@
           <t>Part vacance sur total charges site</t>
         </is>
       </c>
-      <c r="F15" s="45">
+      <c r="F15" s="48">
         <f>IF(D8&gt;0,F13/D8,0)</f>
         <v/>
       </c>
     </row>
     <row r="16" ht="6" customHeight="1"/>
     <row r="17" ht="27.75" customHeight="1">
-      <c r="A17" s="36" t="inlineStr">
+      <c r="A17" s="40" t="inlineStr">
         <is>
           <t>ℹ  QP annuelle = Total site HT × clé de répartition. Coût vacance = QP annuelle × fraction de l'année non occupée.</t>
         </is>

</xml_diff>

<commit_message>
Always include HONORAIRES section in lot tabs for manual entry
Every lot tab now contains a fixed HONORAIRES block (after other categories,
before TOTAL) with an "Honoraires Gestion Technique" row: col D is left empty
for manual entry, col E = 1 (full year), col F = D×E (IF guard avoids #VALUE
when D is empty). The TOTAL formula automatically includes the HONORAIRES
subtotal. The section is skipped if HONORAIRES data is already present in the
input charges to avoid duplication.

https://claude.ai/code/session_016DCHgeFEbekAwEc4Sro4Qi
</commit_message>
<xml_diff>
--- a/regularisation_ORMES_A_2025.xlsx
+++ b/regularisation_ORMES_A_2025.xlsx
@@ -170,7 +170,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -273,6 +273,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -3697,7 +3703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -4326,143 +4332,188 @@
         <v/>
       </c>
     </row>
-    <row r="30" ht="7.55" customHeight="1"/>
-    <row r="31" ht="21.75" customHeight="1">
-      <c r="A31" s="15" t="inlineStr">
+    <row r="30" ht="6" customHeight="1"/>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>HONORAIRES</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="15.05" customHeight="1">
+      <c r="A32" s="31" t="inlineStr">
+        <is>
+          <t>Honoraires Gestion Technique</t>
+        </is>
+      </c>
+      <c r="D32" s="36" t="n"/>
+      <c r="E32" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" s="33">
+        <f>IF(D32="","",D32*E32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="10" t="inlineStr">
+        <is>
+          <t>Sous-total — HONORAIRES</t>
+        </is>
+      </c>
+      <c r="C33" s="11">
+        <f>SUM(C32:C32)</f>
+        <v/>
+      </c>
+      <c r="D33" s="11">
+        <f>SUM(D32:D32)</f>
+        <v/>
+      </c>
+      <c r="E33" s="35" t="n"/>
+      <c r="F33" s="11">
+        <f>SUM(F32:F32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" ht="7.55" customHeight="1"/>
+    <row r="35" ht="21.75" customHeight="1">
+      <c r="A35" s="15" t="inlineStr">
         <is>
           <t>TOTAL CHARGES RÉCUPÉRABLES RÉELLES (€ HT)</t>
         </is>
       </c>
-      <c r="C31" s="16">
-        <f>C9+C12+C26+C29</f>
-        <v/>
-      </c>
-      <c r="D31" s="16">
-        <f>D9+D12+D26+D29</f>
-        <v/>
-      </c>
-      <c r="E31" s="36" t="n"/>
-      <c r="F31" s="16">
-        <f>F9+F12+F26+F29</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32" ht="7.55" customHeight="1"/>
-    <row r="33" ht="19.55" customHeight="1">
-      <c r="A33" s="5" t="inlineStr">
+      <c r="C35" s="16">
+        <f>C9+C12+C26+C29+C33</f>
+        <v/>
+      </c>
+      <c r="D35" s="16">
+        <f>D9+D12+D26+D29+D33</f>
+        <v/>
+      </c>
+      <c r="E35" s="38" t="n"/>
+      <c r="F35" s="16">
+        <f>F9+F12+F26+F29+F33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" ht="7.55" customHeight="1"/>
+    <row r="37" ht="19.55" customHeight="1">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>Provisions pour charges versées</t>
         </is>
       </c>
-      <c r="C33" s="37" t="n"/>
-      <c r="D33" s="27" t="inlineStr">
+      <c r="C37" s="39" t="n"/>
+      <c r="D37" s="27" t="inlineStr">
         <is>
           <t>Montant annuel (€)</t>
         </is>
       </c>
-      <c r="E33" s="37" t="n"/>
-      <c r="F33" s="27" t="inlineStr">
+      <c r="E37" s="39" t="n"/>
+      <c r="F37" s="27" t="inlineStr">
         <is>
           <t>Montant locataire (€)</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="15.8" customHeight="1">
-      <c r="A34" s="21" t="inlineStr">
+    <row r="38" ht="15.8" customHeight="1">
+      <c r="A38" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">  1er trimestre (T1)</t>
         </is>
       </c>
-      <c r="F34" s="33" t="n">
+      <c r="F38" s="33" t="n">
         <v>2990.6</v>
       </c>
     </row>
-    <row r="35" ht="15.8" customHeight="1">
-      <c r="A35" s="21" t="inlineStr">
+    <row r="39" ht="15.8" customHeight="1">
+      <c r="A39" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">  2e trimestre (T2)</t>
         </is>
       </c>
-      <c r="F35" s="33" t="n">
+      <c r="F39" s="33" t="n">
         <v>25284.11</v>
       </c>
     </row>
-    <row r="36" ht="15.8" customHeight="1">
-      <c r="A36" s="21" t="inlineStr">
+    <row r="40" ht="15.8" customHeight="1">
+      <c r="A40" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">  3e trimestre (T3)</t>
         </is>
       </c>
-      <c r="F36" s="33" t="n">
+      <c r="F40" s="33" t="n">
         <v>28376.42</v>
       </c>
     </row>
-    <row r="37" ht="15.8" customHeight="1">
-      <c r="A37" s="21" t="inlineStr">
+    <row r="41" ht="15.8" customHeight="1">
+      <c r="A41" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">  4e trimestre (T4)</t>
         </is>
       </c>
-      <c r="F37" s="33" t="n">
+      <c r="F41" s="33" t="n">
         <v>28376.42</v>
       </c>
     </row>
-    <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="10" t="inlineStr">
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="10" t="inlineStr">
         <is>
           <t>Total provisions pour charges versées →</t>
         </is>
       </c>
-      <c r="D38" s="11">
-        <f>SUM(D34:D37)</f>
-        <v/>
-      </c>
-      <c r="E38" s="35" t="n"/>
-      <c r="F38" s="11">
-        <f>SUM(F34:F37)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39" ht="7.55" customHeight="1"/>
-    <row r="40" ht="21.75" customHeight="1">
-      <c r="A40" s="38">
-        <f>IF(F31-F38&gt;0,"SOLDE DÉBITEUR","SOLDE CRÉDITEUR")</f>
-        <v/>
-      </c>
-      <c r="D40" s="39">
-        <f>D31-D38</f>
-        <v/>
-      </c>
-      <c r="E40" s="37" t="n"/>
-      <c r="F40" s="39">
-        <f>F31-F38</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42" ht="27.75" customHeight="1">
-      <c r="A42" s="40" t="inlineStr">
+      <c r="D42" s="11">
+        <f>SUM(D38:D41)</f>
+        <v/>
+      </c>
+      <c r="E42" s="35" t="n"/>
+      <c r="F42" s="11">
+        <f>SUM(F38:F41)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43" ht="7.55" customHeight="1"/>
+    <row r="44" ht="21.75" customHeight="1">
+      <c r="A44" s="40">
+        <f>IF(F35-F42&gt;0,"SOLDE DÉBITEUR","SOLDE CRÉDITEUR")</f>
+        <v/>
+      </c>
+      <c r="D44" s="41">
+        <f>D35-D42</f>
+        <v/>
+      </c>
+      <c r="E44" s="39" t="n"/>
+      <c r="F44" s="41">
+        <f>F35-F42</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46" ht="27.75" customHeight="1">
+      <c r="A46" s="42" t="inlineStr">
         <is>
           <t>ℹ  Clé répartition = surface lot ÷ surface totale site. Période = nombre de jours d'occupation ÷ 365.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="18">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A26:B26"/>
+    <mergeCell ref="A42:C42"/>
     <mergeCell ref="A10:F10"/>
-    <mergeCell ref="A42:F42"/>
     <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A44:C44"/>
     <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A46:F46"/>
     <mergeCell ref="A33:B33"/>
     <mergeCell ref="A9:B9"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A5:F5"/>
     <mergeCell ref="A27:F27"/>
-    <mergeCell ref="A40:C40"/>
+    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A37:B37"/>
     <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="A35:B35"/>
     <mergeCell ref="A12:B12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4475,7 +4526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -5104,131 +5155,176 @@
         <v/>
       </c>
     </row>
-    <row r="30" ht="7.55" customHeight="1"/>
-    <row r="31" ht="21.75" customHeight="1">
-      <c r="A31" s="15" t="inlineStr">
+    <row r="30" ht="6" customHeight="1"/>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>HONORAIRES</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="15.05" customHeight="1">
+      <c r="A32" s="31" t="inlineStr">
+        <is>
+          <t>Honoraires Gestion Technique</t>
+        </is>
+      </c>
+      <c r="D32" s="36" t="n"/>
+      <c r="E32" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" s="33">
+        <f>IF(D32="","",D32*E32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="10" t="inlineStr">
+        <is>
+          <t>Sous-total — HONORAIRES</t>
+        </is>
+      </c>
+      <c r="C33" s="11">
+        <f>SUM(C32:C32)</f>
+        <v/>
+      </c>
+      <c r="D33" s="11">
+        <f>SUM(D32:D32)</f>
+        <v/>
+      </c>
+      <c r="E33" s="35" t="n"/>
+      <c r="F33" s="11">
+        <f>SUM(F32:F32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" ht="7.55" customHeight="1"/>
+    <row r="35" ht="21.75" customHeight="1">
+      <c r="A35" s="15" t="inlineStr">
         <is>
           <t>TOTAL CHARGES RÉCUPÉRABLES RÉELLES (€ HT)</t>
         </is>
       </c>
-      <c r="C31" s="16">
-        <f>C9+C12+C26+C29</f>
-        <v/>
-      </c>
-      <c r="D31" s="16">
-        <f>D9+D12+D26+D29</f>
-        <v/>
-      </c>
-      <c r="E31" s="36" t="n"/>
-      <c r="F31" s="16">
-        <f>F9+F12+F26+F29</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32" ht="7.55" customHeight="1"/>
-    <row r="33" ht="19.55" customHeight="1">
-      <c r="A33" s="5" t="inlineStr">
+      <c r="C35" s="16">
+        <f>C9+C12+C26+C29+C33</f>
+        <v/>
+      </c>
+      <c r="D35" s="16">
+        <f>D9+D12+D26+D29+D33</f>
+        <v/>
+      </c>
+      <c r="E35" s="38" t="n"/>
+      <c r="F35" s="16">
+        <f>F9+F12+F26+F29+F33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" ht="7.55" customHeight="1"/>
+    <row r="37" ht="19.55" customHeight="1">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>Provisions pour charges versées</t>
         </is>
       </c>
-      <c r="C33" s="37" t="n"/>
-      <c r="D33" s="27" t="inlineStr">
+      <c r="C37" s="39" t="n"/>
+      <c r="D37" s="27" t="inlineStr">
         <is>
           <t>Montant annuel (€)</t>
         </is>
       </c>
-      <c r="E33" s="37" t="n"/>
-      <c r="F33" s="27" t="inlineStr">
+      <c r="E37" s="39" t="n"/>
+      <c r="F37" s="27" t="inlineStr">
         <is>
           <t>Montant locataire (€)</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="15.8" customHeight="1">
-      <c r="A34" s="21" t="inlineStr">
+    <row r="38" ht="15.8" customHeight="1">
+      <c r="A38" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">  1er trimestre (T1)</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="15.8" customHeight="1">
-      <c r="A35" s="21" t="inlineStr">
+    <row r="39" ht="15.8" customHeight="1">
+      <c r="A39" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">  2e trimestre (T2)</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="15.8" customHeight="1">
-      <c r="A36" s="21" t="inlineStr">
+    <row r="40" ht="15.8" customHeight="1">
+      <c r="A40" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">  3e trimestre (T3)</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="15.8" customHeight="1">
-      <c r="A37" s="21" t="inlineStr">
+    <row r="41" ht="15.8" customHeight="1">
+      <c r="A41" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">  4e trimestre (T4)</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="10" t="inlineStr">
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="10" t="inlineStr">
         <is>
           <t>Total provisions pour charges versées →</t>
         </is>
       </c>
-      <c r="D38" s="11">
-        <f>SUM(D34:D37)</f>
-        <v/>
-      </c>
-      <c r="E38" s="35" t="n"/>
-      <c r="F38" s="11">
-        <f>SUM(F34:F37)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39" ht="7.55" customHeight="1"/>
-    <row r="40" ht="21.75" customHeight="1">
-      <c r="A40" s="38">
-        <f>IF(F31-F38&gt;0,"SOLDE DÉBITEUR","SOLDE CRÉDITEUR")</f>
-        <v/>
-      </c>
-      <c r="D40" s="39">
-        <f>D31-D38</f>
-        <v/>
-      </c>
-      <c r="E40" s="37" t="n"/>
-      <c r="F40" s="39">
-        <f>F31-F38</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42" ht="27.75" customHeight="1">
-      <c r="A42" s="40" t="inlineStr">
+      <c r="D42" s="11">
+        <f>SUM(D38:D41)</f>
+        <v/>
+      </c>
+      <c r="E42" s="35" t="n"/>
+      <c r="F42" s="11">
+        <f>SUM(F38:F41)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43" ht="7.55" customHeight="1"/>
+    <row r="44" ht="21.75" customHeight="1">
+      <c r="A44" s="40">
+        <f>IF(F35-F42&gt;0,"SOLDE DÉBITEUR","SOLDE CRÉDITEUR")</f>
+        <v/>
+      </c>
+      <c r="D44" s="41">
+        <f>D35-D42</f>
+        <v/>
+      </c>
+      <c r="E44" s="39" t="n"/>
+      <c r="F44" s="41">
+        <f>F35-F42</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46" ht="27.75" customHeight="1">
+      <c r="A46" s="42" t="inlineStr">
         <is>
           <t>ℹ  Clé répartition = surface lot ÷ surface totale site. Période = nombre de jours d'occupation ÷ 365.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="18">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A26:B26"/>
+    <mergeCell ref="A42:C42"/>
     <mergeCell ref="A10:F10"/>
-    <mergeCell ref="A42:F42"/>
     <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A44:C44"/>
     <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A46:F46"/>
     <mergeCell ref="A33:B33"/>
     <mergeCell ref="A9:B9"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A5:F5"/>
     <mergeCell ref="A27:F27"/>
-    <mergeCell ref="A40:C40"/>
+    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A37:B37"/>
     <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="A35:B35"/>
     <mergeCell ref="A12:B12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5300,7 +5396,7 @@
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="41">
+      <c r="A5" s="43">
         <f>Paramètres!A7</f>
         <v/>
       </c>
@@ -5308,12 +5404,12 @@
         <f>Paramètres!B7</f>
         <v/>
       </c>
-      <c r="C5" s="42">
+      <c r="C5" s="44">
         <f>Paramètres!C7</f>
         <v/>
       </c>
       <c r="D5" s="33">
-        <f>'C1 C2'!D31</f>
+        <f>'C1 C2'!D35</f>
         <v/>
       </c>
       <c r="E5" s="34">
@@ -5321,12 +5417,12 @@
         <v/>
       </c>
       <c r="F5" s="29">
-        <f>IF(Paramètres!B7="Vacant",'C1 C2'!D31,'C1 C2'!D31-'C1 C2'!F31)</f>
+        <f>IF(Paramètres!B7="Vacant",'C1 C2'!D35,'C1 C2'!D35-'C1 C2'!F35)</f>
         <v/>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="41">
+      <c r="A6" s="43">
         <f>Paramètres!A8</f>
         <v/>
       </c>
@@ -5334,12 +5430,12 @@
         <f>Paramètres!B8</f>
         <v/>
       </c>
-      <c r="C6" s="42">
+      <c r="C6" s="44">
         <f>Paramètres!C8</f>
         <v/>
       </c>
       <c r="D6" s="33">
-        <f>'C3 C4 C5'!D31</f>
+        <f>'C3 C4 C5'!D35</f>
         <v/>
       </c>
       <c r="E6" s="34">
@@ -5347,7 +5443,7 @@
         <v/>
       </c>
       <c r="F6" s="29">
-        <f>IF(Paramètres!B8="Vacant",'C3 C4 C5'!D31,'C3 C4 C5'!D31-'C3 C4 C5'!F31)</f>
+        <f>IF(Paramètres!B8="Vacant",'C3 C4 C5'!D35,'C3 C4 C5'!D35-'C3 C4 C5'!F35)</f>
         <v/>
       </c>
     </row>
@@ -5371,7 +5467,7 @@
           <t>Nombre de lots vacants</t>
         </is>
       </c>
-      <c r="D9" s="43">
+      <c r="D9" s="45">
         <f>COUNTIF(B5:B6,"Vacant")</f>
         <v/>
       </c>
@@ -5380,24 +5476,24 @@
     </row>
     <row r="10" ht="6" customHeight="1"/>
     <row r="11" ht="19.55" customHeight="1">
-      <c r="A11" s="44" t="inlineStr">
+      <c r="A11" s="46" t="inlineStr">
         <is>
           <t>Charges non récupérables (Frais Bancaires + CAPEX)</t>
         </is>
       </c>
-      <c r="F11" s="45">
+      <c r="F11" s="47">
         <f>'Récapitulatif 2025'!E118</f>
         <v/>
       </c>
     </row>
     <row r="12" ht="6" customHeight="1"/>
     <row r="13" ht="25.55" customHeight="1">
-      <c r="A13" s="46" t="inlineStr">
+      <c r="A13" s="48" t="inlineStr">
         <is>
           <t>TOTAL COÛT DE LA VACANCE LOCATIVE (€ HT)</t>
         </is>
       </c>
-      <c r="F13" s="47">
+      <c r="F13" s="49">
         <f>F5+F6+F11</f>
         <v/>
       </c>
@@ -5409,14 +5505,14 @@
           <t>Part vacance sur total charges site</t>
         </is>
       </c>
-      <c r="F15" s="48">
+      <c r="F15" s="50">
         <f>IF(D8&gt;0,F13/D8,0)</f>
         <v/>
       </c>
     </row>
     <row r="16" ht="6" customHeight="1"/>
     <row r="17" ht="27.75" customHeight="1">
-      <c r="A17" s="40" t="inlineStr">
+      <c r="A17" s="42" t="inlineStr">
         <is>
           <t>ℹ  QP annuelle = Total site HT × clé de répartition. Coût vacance = QP annuelle × fraction de l'année non occupée.</t>
         </is>

</xml_diff>